<commit_message>
Add script for setting up data and initial sample sheet
</commit_message>
<xml_diff>
--- a/sample_sheet.xlsx
+++ b/sample_sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/cluster-gjb_lab/jabbott/Projects/JCA_NRSW_Compost/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{344F5EEC-EAC2-0F42-9EDE-8840881DF874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78513DD1-1597-C841-8703-54681BAFE6BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{EC14CA74-949E-9541-9E2A-AB04829A19E1}"/>
   </bookViews>
@@ -122,9 +122,6 @@
     <t>¬∫C</t>
   </si>
   <si>
-    <t>NRS2102 </t>
-  </si>
-  <si>
     <t>\\estorage.dundee.ac.uk\cluster\nrsw_lab\nrstanleywall\compost_isolates\230727_NGS\rawdata</t>
   </si>
   <si>
@@ -143,81 +140,12 @@
     <t>Edinburgh Botanic Gardens</t>
   </si>
   <si>
-    <t>NRS2103 </t>
-  </si>
-  <si>
     <t>\\estorage.dundee.ac.uk\cluster\nrsw_lab\nrstanleywall\20251016_compost_hybrid\rawdata_long</t>
   </si>
   <si>
-    <t>NRS2104 </t>
-  </si>
-  <si>
     <t>\\estorage.dundee.ac.uk\cluster\nrsw_lab\nrstanleywall\compost_isolates\230801_NGS\rawdata</t>
   </si>
   <si>
-    <t>NRS2105 </t>
-  </si>
-  <si>
-    <t>NRS2106 </t>
-  </si>
-  <si>
-    <t>NRS2107 </t>
-  </si>
-  <si>
-    <t>NRS2108 </t>
-  </si>
-  <si>
-    <t>NRS2109 </t>
-  </si>
-  <si>
-    <t>NRS2110 </t>
-  </si>
-  <si>
-    <t>NRS2111 </t>
-  </si>
-  <si>
-    <t>NRS2113 </t>
-  </si>
-  <si>
-    <t>NRS2114 </t>
-  </si>
-  <si>
-    <t>NRS2125 </t>
-  </si>
-  <si>
-    <t>NRS2128 </t>
-  </si>
-  <si>
-    <t>NRS2130 </t>
-  </si>
-  <si>
-    <t>NRS2131 </t>
-  </si>
-  <si>
-    <t>NRS2132 </t>
-  </si>
-  <si>
-    <t>NRS2133 </t>
-  </si>
-  <si>
-    <t>NRS2135 </t>
-  </si>
-  <si>
-    <t>NRS2136 </t>
-  </si>
-  <si>
-    <t>NRS2137 </t>
-  </si>
-  <si>
-    <t>NRS2139 </t>
-  </si>
-  <si>
-    <t>NRS2140 </t>
-  </si>
-  <si>
-    <t>NRS6072 </t>
-  </si>
-  <si>
     <t>10.1099/mic.0.001082</t>
   </si>
   <si>
@@ -233,9 +161,6 @@
     <t>Mesagros, Greece</t>
   </si>
   <si>
-    <t>NRS6077 </t>
-  </si>
-  <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242198_NRS6077_1.fastq.gz</t>
   </si>
   <si>
@@ -245,9 +170,6 @@
     <t>Myrsinis, Greece</t>
   </si>
   <si>
-    <t>NRS6080 </t>
-  </si>
-  <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242193_NRS6080_1.fastq.gz</t>
   </si>
   <si>
@@ -263,9 +185,6 @@
     <t>open environment</t>
   </si>
   <si>
-    <t>NRS6082 </t>
-  </si>
-  <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242199_NRS6082_1.fastq.gz</t>
   </si>
   <si>
@@ -278,9 +197,6 @@
     <t>Glenshee, Blairgrowrie, Scotland, UK</t>
   </si>
   <si>
-    <t>NRS6095 </t>
-  </si>
-  <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242200_NRS6095_1.fastq.gz</t>
   </si>
   <si>
@@ -296,18 +212,12 @@
     <t>garden</t>
   </si>
   <si>
-    <t>NRS6101 </t>
-  </si>
-  <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242194_NRS6101_1.fastq.gz</t>
   </si>
   <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242194_NRS6101_2.fastq.gz</t>
   </si>
   <si>
-    <t>NRS6104 </t>
-  </si>
-  <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242195_NRS6104_1.fastq.gz</t>
   </si>
   <si>
@@ -317,9 +227,6 @@
     <t xml:space="preserve"> in raised vegetable bed</t>
   </si>
   <si>
-    <t>NRS6106 </t>
-  </si>
-  <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242196_NRS6106_1.fastq.gz</t>
   </si>
   <si>
@@ -329,9 +236,6 @@
     <t>vegetable garden soil</t>
   </si>
   <si>
-    <t>NRS6112 </t>
-  </si>
-  <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242197_NRS6112_1.fastq.gz</t>
   </si>
   <si>
@@ -341,18 +245,12 @@
     <t>mature deciduous trees present</t>
   </si>
   <si>
-    <t>NRS6115 </t>
-  </si>
-  <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242201_NRS6115_1.fastq.gz</t>
   </si>
   <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242201_NRS6115_2.fastq.gz</t>
   </si>
   <si>
-    <t>NRS6119 </t>
-  </si>
-  <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242202_NRS6119_1.fastq.gz</t>
   </si>
   <si>
@@ -362,9 +260,6 @@
     <t xml:space="preserve">potato patch in rear garden </t>
   </si>
   <si>
-    <t>NRS6133 </t>
-  </si>
-  <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242203_NRS6133_1.fastq.gz</t>
   </si>
   <si>
@@ -374,27 +269,18 @@
     <t>allotment garden</t>
   </si>
   <si>
-    <t>NRS6136 </t>
-  </si>
-  <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242204_NRS6136_1.fastq.gz</t>
   </si>
   <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242204_NRS6136_2.fastq.gz</t>
   </si>
   <si>
-    <t>NRS6149 </t>
-  </si>
-  <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242205_NRS6149_1.fastq.gz</t>
   </si>
   <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242205_NRS6149_2.fastq.gz</t>
   </si>
   <si>
-    <t>NRS6150 </t>
-  </si>
-  <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242206_NRS6150_1.fastq.gz</t>
   </si>
   <si>
@@ -404,18 +290,12 @@
     <t>compost</t>
   </si>
   <si>
-    <t>NRS6166 </t>
-  </si>
-  <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242207_NRS6166_1.fastq.gz</t>
   </si>
   <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242207_NRS6166_2.fastq.gz</t>
   </si>
   <si>
-    <t>NRS6212 </t>
-  </si>
-  <si>
     <t>https://microbesng-data.s3-eu-west-1.amazonaws.com/projects/e549fa4e70_20221108_StanleyWall1/242208_NRS6212_1.fastq.gz</t>
   </si>
   <si>
@@ -423,6 +303,126 @@
   </si>
   <si>
     <t xml:space="preserve"> livestock present</t>
+  </si>
+  <si>
+    <t>NRS2102</t>
+  </si>
+  <si>
+    <t>NRS2103</t>
+  </si>
+  <si>
+    <t>NRS2104</t>
+  </si>
+  <si>
+    <t>NRS2105</t>
+  </si>
+  <si>
+    <t>NRS2106</t>
+  </si>
+  <si>
+    <t>NRS2107</t>
+  </si>
+  <si>
+    <t>NRS2108</t>
+  </si>
+  <si>
+    <t>NRS2109</t>
+  </si>
+  <si>
+    <t>NRS2110</t>
+  </si>
+  <si>
+    <t>NRS2111</t>
+  </si>
+  <si>
+    <t>NRS2113</t>
+  </si>
+  <si>
+    <t>NRS2114</t>
+  </si>
+  <si>
+    <t>NRS2125</t>
+  </si>
+  <si>
+    <t>NRS2128</t>
+  </si>
+  <si>
+    <t>NRS2130</t>
+  </si>
+  <si>
+    <t>NRS2131</t>
+  </si>
+  <si>
+    <t>NRS2132</t>
+  </si>
+  <si>
+    <t>NRS2133</t>
+  </si>
+  <si>
+    <t>NRS2135</t>
+  </si>
+  <si>
+    <t>NRS2136</t>
+  </si>
+  <si>
+    <t>NRS2137</t>
+  </si>
+  <si>
+    <t>NRS2139</t>
+  </si>
+  <si>
+    <t>NRS2140</t>
+  </si>
+  <si>
+    <t>NRS6072</t>
+  </si>
+  <si>
+    <t>NRS6077</t>
+  </si>
+  <si>
+    <t>NRS6080</t>
+  </si>
+  <si>
+    <t>NRS6082</t>
+  </si>
+  <si>
+    <t>NRS6095</t>
+  </si>
+  <si>
+    <t>NRS6101</t>
+  </si>
+  <si>
+    <t>NRS6104</t>
+  </si>
+  <si>
+    <t>NRS6106</t>
+  </si>
+  <si>
+    <t>NRS6112</t>
+  </si>
+  <si>
+    <t>NRS6115</t>
+  </si>
+  <si>
+    <t>NRS6119</t>
+  </si>
+  <si>
+    <t>NRS6133</t>
+  </si>
+  <si>
+    <t>NRS6136</t>
+  </si>
+  <si>
+    <t>NRS6149</t>
+  </si>
+  <si>
+    <t>NRS6150</t>
+  </si>
+  <si>
+    <t>NRS6166</t>
+  </si>
+  <si>
+    <t>NRS6212</t>
   </si>
 </sst>
 </file>
@@ -1481,18 +1481,18 @@
     </row>
     <row r="4" spans="1:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C4" s="2" t="s">
-        <v>28</v>
+        <v>89</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F4" s="2"/>
       <c r="J4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q4" s="3">
         <v>44956</v>
@@ -1504,13 +1504,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U4" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U4" s="7" t="s">
+      <c r="V4" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V4" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W4" s="1">
         <v>52</v>
@@ -1518,21 +1518,21 @@
     </row>
     <row r="5" spans="1:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C5" s="2" t="s">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K5" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q5" s="3">
         <v>44956</v>
@@ -1544,13 +1544,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U5" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U5" s="7" t="s">
+      <c r="V5" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V5" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W5" s="1">
         <v>52</v>
@@ -1558,17 +1558,17 @@
     </row>
     <row r="6" spans="1:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C6" s="2" t="s">
-        <v>37</v>
+        <v>91</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q6" s="3">
         <v>44956</v>
@@ -1580,13 +1580,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U6" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U6" s="7" t="s">
+      <c r="V6" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V6" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W6" s="1">
         <v>52</v>
@@ -1594,18 +1594,18 @@
     </row>
     <row r="7" spans="1:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C7" s="2" t="s">
-        <v>39</v>
+        <v>92</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F7" s="2"/>
       <c r="J7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K7" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q7" s="3">
         <v>44956</v>
@@ -1617,13 +1617,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U7" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U7" s="7" t="s">
+      <c r="V7" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W7" s="1">
         <v>52</v>
@@ -1631,21 +1631,21 @@
     </row>
     <row r="8" spans="1:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C8" s="2" t="s">
-        <v>40</v>
+        <v>93</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K8" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q8" s="3">
         <v>44956</v>
@@ -1657,13 +1657,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U8" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U8" s="7" t="s">
+      <c r="V8" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V8" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W8" s="1">
         <v>52</v>
@@ -1671,20 +1671,20 @@
     </row>
     <row r="9" spans="1:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C9" s="2" t="s">
-        <v>41</v>
+        <v>94</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K9" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q9" s="3">
         <v>44956</v>
@@ -1696,13 +1696,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U9" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U9" s="7" t="s">
+      <c r="V9" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V9" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W9" s="1">
         <v>52</v>
@@ -1710,20 +1710,20 @@
     </row>
     <row r="10" spans="1:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C10" s="2" t="s">
-        <v>42</v>
+        <v>95</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K10" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q10" s="3">
         <v>44956</v>
@@ -1735,13 +1735,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U10" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U10" s="7" t="s">
+      <c r="V10" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V10" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W10" s="1">
         <v>52</v>
@@ -1749,20 +1749,20 @@
     </row>
     <row r="11" spans="1:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C11" s="2" t="s">
-        <v>43</v>
+        <v>96</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K11" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q11" s="3">
         <v>44956</v>
@@ -1774,13 +1774,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U11" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U11" s="7" t="s">
+      <c r="V11" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V11" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W11" s="1">
         <v>52</v>
@@ -1788,17 +1788,17 @@
     </row>
     <row r="12" spans="1:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C12" s="2" t="s">
-        <v>44</v>
+        <v>97</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K12" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K12" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q12" s="3">
         <v>44956</v>
@@ -1810,13 +1810,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U12" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U12" s="7" t="s">
+      <c r="V12" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V12" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W12" s="1">
         <v>52</v>
@@ -1824,17 +1824,17 @@
     </row>
     <row r="13" spans="1:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C13" s="2" t="s">
-        <v>45</v>
+        <v>98</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K13" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K13" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q13" s="3">
         <v>44956</v>
@@ -1846,13 +1846,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T13" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U13" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U13" s="7" t="s">
+      <c r="V13" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V13" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W13" s="1">
         <v>52</v>
@@ -1860,18 +1860,18 @@
     </row>
     <row r="14" spans="1:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C14" s="2" t="s">
-        <v>46</v>
+        <v>99</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F14" s="2"/>
       <c r="J14" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K14" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q14" s="3">
         <v>44956</v>
@@ -1883,13 +1883,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U14" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U14" s="7" t="s">
+      <c r="V14" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V14" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W14" s="1">
         <v>14</v>
@@ -1897,18 +1897,18 @@
     </row>
     <row r="15" spans="1:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C15" s="2" t="s">
-        <v>47</v>
+        <v>100</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F15" s="2"/>
       <c r="J15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K15" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K15" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q15" s="3">
         <v>44956</v>
@@ -1920,13 +1920,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T15" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U15" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U15" s="7" t="s">
+      <c r="V15" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V15" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W15" s="1">
         <v>14</v>
@@ -1934,21 +1934,21 @@
     </row>
     <row r="16" spans="1:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C16" s="2" t="s">
-        <v>48</v>
+        <v>101</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J16" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K16" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K16" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q16" s="3">
         <v>44956</v>
@@ -1960,13 +1960,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T16" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U16" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U16" s="7" t="s">
+      <c r="V16" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V16" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W16" s="1">
         <v>25</v>
@@ -1974,18 +1974,18 @@
     </row>
     <row r="17" spans="3:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C17" s="2" t="s">
-        <v>49</v>
+        <v>102</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F17" s="2"/>
       <c r="J17" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K17" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K17" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q17" s="3">
         <v>44956</v>
@@ -1997,13 +1997,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T17" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U17" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U17" s="7" t="s">
+      <c r="V17" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V17" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W17" s="1">
         <v>25</v>
@@ -2011,18 +2011,18 @@
     </row>
     <row r="18" spans="3:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C18" s="2" t="s">
-        <v>50</v>
+        <v>103</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F18" s="2"/>
       <c r="J18" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K18" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K18" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q18" s="3">
         <v>44956</v>
@@ -2034,13 +2034,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T18" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U18" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U18" s="7" t="s">
+      <c r="V18" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V18" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W18" s="1">
         <v>25</v>
@@ -2048,18 +2048,18 @@
     </row>
     <row r="19" spans="3:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C19" s="2" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="D19" s="2"/>
       <c r="E19" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F19" s="2"/>
       <c r="J19" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K19" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K19" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q19" s="3">
         <v>44956</v>
@@ -2071,13 +2071,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T19" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U19" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U19" s="7" t="s">
+      <c r="V19" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V19" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W19" s="1">
         <v>52</v>
@@ -2085,20 +2085,20 @@
     </row>
     <row r="20" spans="3:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C20" s="2" t="s">
-        <v>52</v>
+        <v>105</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J20" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K20" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K20" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q20" s="3">
         <v>44956</v>
@@ -2110,13 +2110,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T20" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U20" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U20" s="7" t="s">
+      <c r="V20" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V20" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W20" s="1">
         <v>52</v>
@@ -2124,17 +2124,17 @@
     </row>
     <row r="21" spans="3:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C21" s="2" t="s">
-        <v>53</v>
+        <v>106</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J21" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K21" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K21" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q21" s="3">
         <v>44956</v>
@@ -2146,13 +2146,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T21" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U21" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U21" s="7" t="s">
+      <c r="V21" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V21" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W21" s="1">
         <v>52</v>
@@ -2160,18 +2160,18 @@
     </row>
     <row r="22" spans="3:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C22" s="2" t="s">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F22" s="2"/>
       <c r="J22" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K22" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K22" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q22" s="3">
         <v>44956</v>
@@ -2183,13 +2183,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T22" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U22" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U22" s="7" t="s">
+      <c r="V22" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V22" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W22" s="1">
         <v>52</v>
@@ -2197,20 +2197,20 @@
     </row>
     <row r="23" spans="3:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C23" s="2" t="s">
-        <v>55</v>
+        <v>108</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J23" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K23" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K23" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q23" s="3">
         <v>44956</v>
@@ -2222,13 +2222,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T23" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U23" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U23" s="7" t="s">
+      <c r="V23" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V23" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W23" s="1">
         <v>52</v>
@@ -2236,17 +2236,17 @@
     </row>
     <row r="24" spans="3:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C24" s="2" t="s">
-        <v>56</v>
+        <v>109</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J24" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K24" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K24" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q24" s="3">
         <v>44956</v>
@@ -2258,13 +2258,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T24" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U24" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U24" s="7" t="s">
+      <c r="V24" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V24" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W24" s="1">
         <v>52</v>
@@ -2272,17 +2272,17 @@
     </row>
     <row r="25" spans="3:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C25" s="2" t="s">
-        <v>57</v>
+        <v>110</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J25" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K25" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K25" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q25" s="3">
         <v>44956</v>
@@ -2294,13 +2294,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T25" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U25" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U25" s="7" t="s">
+      <c r="V25" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V25" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W25" s="1">
         <v>52</v>
@@ -2308,17 +2308,17 @@
     </row>
     <row r="26" spans="3:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C26" s="2" t="s">
-        <v>58</v>
+        <v>111</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J26" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K26" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K26" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q26" s="3">
         <v>44956</v>
@@ -2330,13 +2330,13 @@
         <v>-3.2126426159313399</v>
       </c>
       <c r="T26" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U26" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="U26" s="7" t="s">
+      <c r="V26" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="V26" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="W26" s="1">
         <v>52</v>
@@ -2344,22 +2344,22 @@
     </row>
     <row r="27" spans="3:23" s="8" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C27" s="8" t="s">
-        <v>59</v>
+        <v>112</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="J27" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K27" s="8" t="s">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="Q27" s="11">
         <v>42872</v>
@@ -2371,30 +2371,30 @@
         <v>23.516715059188002</v>
       </c>
       <c r="T27" s="8" t="s">
-        <v>64</v>
+        <v>40</v>
       </c>
     </row>
     <row r="28" spans="3:23" s="8" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C28" s="8" t="s">
-        <v>65</v>
+        <v>113</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>66</v>
+        <v>41</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K28" s="8" t="s">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="Q28" s="11">
         <v>42872</v>
@@ -2406,27 +2406,27 @@
         <v>21.2368286335251</v>
       </c>
       <c r="T28" s="8" t="s">
-        <v>68</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" spans="3:23" s="8" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C29" s="8" t="s">
-        <v>69</v>
+        <v>114</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>70</v>
+        <v>44</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>71</v>
+        <v>45</v>
       </c>
       <c r="J29" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K29" s="8" t="s">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="Q29" s="11">
         <v>42878</v>
@@ -2438,36 +2438,36 @@
         <v>-3.3628259981933</v>
       </c>
       <c r="T29" s="8" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="U29" s="8" t="s">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="V29" s="8" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30" spans="3:23" s="8" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C30" s="8" t="s">
-        <v>75</v>
+        <v>115</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J30" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K30" s="8" t="s">
-        <v>78</v>
+        <v>51</v>
       </c>
       <c r="Q30" s="11">
         <v>42878</v>
@@ -2479,33 +2479,33 @@
         <v>-3.4047510435243802</v>
       </c>
       <c r="T30" s="8" t="s">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="U30" s="8" t="s">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="V30" s="8" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" spans="3:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C31" s="1" t="s">
-        <v>80</v>
+        <v>116</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>81</v>
+        <v>53</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K31" s="7" t="s">
-        <v>78</v>
+        <v>51</v>
       </c>
       <c r="Q31" s="3">
         <v>42911</v>
@@ -2517,36 +2517,36 @@
         <v>-2.87724257864217</v>
       </c>
       <c r="T31" s="1" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="U31" s="7" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="V31" s="1" t="s">
-        <v>85</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32" spans="3:23" ht="14" x14ac:dyDescent="0.2">
       <c r="C32" s="1" t="s">
-        <v>86</v>
+        <v>117</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K32" s="7" t="s">
-        <v>78</v>
+        <v>51</v>
       </c>
       <c r="Q32" s="3">
         <v>42911</v>
@@ -2558,33 +2558,33 @@
         <v>-2.87724257864217</v>
       </c>
       <c r="T32" s="1" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="U32" s="7" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="V32" s="1" t="s">
-        <v>85</v>
+        <v>57</v>
       </c>
     </row>
     <row r="33" spans="3:22" ht="14" x14ac:dyDescent="0.2">
       <c r="C33" s="1" t="s">
-        <v>89</v>
+        <v>118</v>
       </c>
       <c r="D33" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E33" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="E33" s="5" t="s">
-        <v>90</v>
-      </c>
       <c r="F33" s="5" t="s">
-        <v>91</v>
+        <v>61</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K33" s="7" t="s">
-        <v>78</v>
+        <v>51</v>
       </c>
       <c r="Q33" s="3">
         <v>42911</v>
@@ -2596,33 +2596,33 @@
         <v>-2.8813236000435598</v>
       </c>
       <c r="T33" s="1" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="U33" s="7" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="V33" s="1" t="s">
-        <v>92</v>
+        <v>62</v>
       </c>
     </row>
     <row r="34" spans="3:22" ht="14" x14ac:dyDescent="0.2">
       <c r="C34" s="1" t="s">
-        <v>93</v>
+        <v>119</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>94</v>
+        <v>63</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>95</v>
+        <v>64</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K34" s="7" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="Q34" s="3">
         <v>42911</v>
@@ -2634,33 +2634,33 @@
         <v>-2.87724257864217</v>
       </c>
       <c r="T34" s="1" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="U34" s="7" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="V34" s="1" t="s">
-        <v>92</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35" spans="3:22" ht="14" x14ac:dyDescent="0.2">
       <c r="C35" s="1" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>98</v>
+        <v>66</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>99</v>
+        <v>67</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K35" s="7" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="Q35" s="3">
         <v>42911</v>
@@ -2672,33 +2672,33 @@
         <v>-2.87724257864217</v>
       </c>
       <c r="T35" s="1" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="U35" s="7" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="V35" s="1" t="s">
-        <v>100</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36" spans="3:22" ht="14" x14ac:dyDescent="0.2">
       <c r="C36" s="1" t="s">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>102</v>
+        <v>69</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>103</v>
+        <v>70</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K36" s="7" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="Q36" s="3">
         <v>42911</v>
@@ -2710,33 +2710,33 @@
         <v>-2.87724257864217</v>
       </c>
       <c r="T36" s="1" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="U36" s="7" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="V36" s="1" t="s">
-        <v>92</v>
+        <v>62</v>
       </c>
     </row>
     <row r="37" spans="3:22" ht="14" x14ac:dyDescent="0.2">
       <c r="C37" s="1" t="s">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>105</v>
+        <v>71</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>106</v>
+        <v>72</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K37" s="7" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="Q37" s="3">
         <v>42911</v>
@@ -2748,33 +2748,33 @@
         <v>-2.87724257864217</v>
       </c>
       <c r="T37" s="1" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="U37" s="7" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="V37" s="1" t="s">
-        <v>107</v>
+        <v>73</v>
       </c>
     </row>
     <row r="38" spans="3:22" ht="14" x14ac:dyDescent="0.2">
       <c r="C38" s="1" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>110</v>
+        <v>75</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K38" s="7" t="s">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="L38" s="7"/>
       <c r="Q38" s="3">
@@ -2787,33 +2787,33 @@
         <v>-2.87724257864217</v>
       </c>
       <c r="T38" s="1" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="U38" s="7" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="V38" s="1" t="s">
-        <v>92</v>
+        <v>62</v>
       </c>
     </row>
     <row r="39" spans="3:22" ht="14" x14ac:dyDescent="0.2">
       <c r="C39" s="1" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>114</v>
+        <v>78</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K39" s="7" t="s">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="Q39" s="3">
         <v>42911</v>
@@ -2825,36 +2825,36 @@
         <v>-2.8813236000435598</v>
       </c>
       <c r="T39" s="1" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="U39" s="7" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="V39" s="1" t="s">
-        <v>92</v>
+        <v>62</v>
       </c>
     </row>
     <row r="40" spans="3:22" ht="14" x14ac:dyDescent="0.2">
       <c r="C40" s="1" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>116</v>
+        <v>79</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>117</v>
+        <v>80</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K40" s="7" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="Q40" s="3">
         <v>42911</v>
@@ -2866,33 +2866,33 @@
         <v>-2.87724257864217</v>
       </c>
       <c r="T40" s="1" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="U40" s="7" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="V40" s="1" t="s">
-        <v>85</v>
+        <v>57</v>
       </c>
     </row>
     <row r="41" spans="3:22" ht="14" x14ac:dyDescent="0.2">
       <c r="C41" s="1" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>119</v>
+        <v>81</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>120</v>
+        <v>82</v>
       </c>
       <c r="J41" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K41" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K41" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q41" s="3">
         <v>42911</v>
@@ -2904,33 +2904,33 @@
         <v>-2.8813236000435598</v>
       </c>
       <c r="T41" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="U41" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="V41" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="U41" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="V41" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="42" spans="3:22" ht="14" x14ac:dyDescent="0.2">
       <c r="C42" s="1" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>123</v>
+        <v>84</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>124</v>
+        <v>85</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K42" s="7" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="Q42" s="3">
         <v>42911</v>
@@ -2942,33 +2942,33 @@
         <v>-2.87724257864217</v>
       </c>
       <c r="T42" s="1" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="U42" s="7" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="V42" s="1" t="s">
-        <v>85</v>
+        <v>57</v>
       </c>
     </row>
     <row r="43" spans="3:22" ht="14" x14ac:dyDescent="0.2">
       <c r="C43" s="1" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K43" s="7" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="Q43" s="3">
         <v>42911</v>
@@ -2980,13 +2980,13 @@
         <v>-2.87724257864217</v>
       </c>
       <c r="T43" s="1" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="U43" s="7" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="V43" s="1" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="52" spans="9:10" x14ac:dyDescent="0.2">

</xml_diff>